<commit_message>
Fix compact win result formula
</commit_message>
<xml_diff>
--- a/ExcelTable/GameString.xlsx
+++ b/ExcelTable/GameString.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rf09e35b159c34e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rab782a655fa04ea4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -657,7 +657,7 @@
         <x:v>208</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>x {0} = {1}</x:v>
+        <x:v>x {0}</x:v>
       </x:c>
     </x:row>
     <x:row r="44">

</xml_diff>

<commit_message>
Add 777 bonus slot trigger
</commit_message>
<xml_diff>
--- a/ExcelTable/GameString.xlsx
+++ b/ExcelTable/GameString.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rab782a655fa04ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rf8b46dd9b83b4e7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -668,6 +668,14 @@
         <x:v> = {0}</x:v>
       </x:c>
     </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="n">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>777 보너스 {0}회 / +{1}</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Redesign top currency HUD
</commit_message>
<xml_diff>
--- a/ExcelTable/GameString.xlsx
+++ b/ExcelTable/GameString.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rf8b46dd9b83b4e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameString" sheetId="1" r:id="Rd5c98c629a4940f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -609,7 +609,7 @@
         <x:v>202</x:v>
       </x:c>
       <x:c r="B37" s="14" t="str">
-        <x:v>프리미엄 {0}</x:v>
+        <x:v>{0}</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -617,7 +617,7 @@
         <x:v>203</x:v>
       </x:c>
       <x:c r="B38" s="14" t="str">
-        <x:v>일반 {0}</x:v>
+        <x:v>{0}</x:v>
       </x:c>
     </x:row>
     <x:row r="39">

</xml_diff>